<commit_message>
[Data] 바뀐 Enemy Data 파싱(Excel -> Json)
</commit_message>
<xml_diff>
--- a/Assets/06 Data/ExcelData/dt_enemy_base_stats.xlsx
+++ b/Assets/06 Data/ExcelData/dt_enemy_base_stats.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Genie\Desktop\duckov-clone\Assets\06 Data\ExcelData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StudyUnity\Duckov\Assets\06 Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC6BE87-D45B-42BA-92B8-6BAC3010A8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64499E6E-8961-4545-BC25-7EC6EFF6F488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-660" yWindow="2685" windowWidth="24300" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30690" yWindow="4155" windowWidth="16005" windowHeight="6075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>uint</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -51,10 +51,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>PatrolRange</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>SightDistance</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -76,10 +72,6 @@
   </si>
   <si>
     <t>시야 거리(m)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>순찰 반경(m)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
@@ -118,7 +110,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -154,13 +146,6 @@
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -217,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -232,9 +217,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -517,38 +499,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>15</v>
@@ -556,11 +537,8 @@
       <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -577,19 +555,16 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>18</v>
-      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -606,19 +581,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>80</v>
       </c>
@@ -632,36 +604,31 @@
         <v>20</v>
       </c>
       <c r="E4" s="4">
-        <v>20</v>
-      </c>
-      <c r="F4" s="4">
         <v>120</v>
       </c>
-      <c r="G4" s="5">
+      <c r="F4" s="5">
         <v>1.2</v>
       </c>
+      <c r="G4" s="4">
+        <v>5</v>
+      </c>
       <c r="H4" s="4">
-        <v>5</v>
-      </c>
-      <c r="I4" s="4">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>